<commit_message>
Store latest works catalogue workbook
</commit_message>
<xml_diff>
--- a/data/List of Works_CHUNG Seung Jae 2.xlsx
+++ b/data/List of Works_CHUNG Seung Jae 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sjchung/Dropbox/My Scores/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\junra\Dropbox\My Scores\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B4828FE-B517-9C4C-9C72-ED6B48C9E06E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1889017-C8B4-49C8-842E-16CD0630D79E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23240" yWindow="5260" windowWidth="29040" windowHeight="15720" xr2:uid="{2CB730A6-55DF-4934-B98A-B96666FCC508}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{2CB730A6-55DF-4934-B98A-B96666FCC508}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="273">
   <si>
     <t>작품명</t>
   </si>
@@ -78,9 +78,6 @@
   </si>
   <si>
     <t>Divertimento for Winds Instruments</t>
-  </si>
-  <si>
-    <t>Das hohepriesterliche Gebet for a cappella</t>
   </si>
   <si>
     <t>In Memoriam Ilhan Yu for Tenor, Horn Quartet and String Quartet</t>
@@ -190,18 +187,10 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>The Dragonfly before the Sun</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Untitleds; Silence Is So Accurate for Viola and Piano</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>Das hohepriesterliche Gebet für Chor</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Stillness in Movement for Bassoon and Piano</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -273,9 +262,6 @@
     <t>2012.01.14</t>
   </si>
   <si>
-    <t>2011.11.27</t>
-  </si>
-  <si>
     <t>2011.10.07</t>
   </si>
   <si>
@@ -303,9 +289,6 @@
     <t>2008.09.16</t>
   </si>
   <si>
-    <t>2007.10.28</t>
-  </si>
-  <si>
     <t>2007.11.09</t>
   </si>
   <si>
@@ -313,9 +296,6 @@
   </si>
   <si>
     <t>2007.05.13</t>
-  </si>
-  <si>
-    <t>2007.02.26</t>
   </si>
   <si>
     <t>2006.12.18</t>
@@ -949,24 +929,52 @@
   </si>
   <si>
     <t>6'</t>
+  </si>
+  <si>
+    <t>2000(Rev. 2007)</t>
+  </si>
+  <si>
+    <t>Yim for Soprano and Tape</t>
+  </si>
+  <si>
+    <t>Soprano, Electronics</t>
+  </si>
+  <si>
+    <t>Das hohepriesterliche Gebet für a Cappella</t>
+  </si>
+  <si>
+    <t>Two Korean Melodies for Piano Solo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Solo</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Piano</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The Flight of the Dragonfly before the Sun</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -974,7 +982,7 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -989,7 +997,7 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -997,7 +1005,7 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1006,7 +1014,7 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1014,7 +1022,7 @@
     <font>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1023,14 +1031,14 @@
       <b/>
       <sz val="10"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1038,7 +1046,7 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1047,7 +1055,7 @@
       <u/>
       <sz val="10"/>
       <color theme="10"/>
-      <name val="Aptos Narrow"/>
+      <name val="맑은 고딕"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1264,8 +1272,8 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="하이퍼링크" xfId="1" builtinId="8"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1281,7 +1289,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1601,18 +1609,18 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:G87"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="54.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" style="5" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" style="2" customWidth="1"/>
-    <col min="4" max="4" width="45.6640625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="8.83203125" style="2"/>
+    <col min="1" max="1" width="54.625" style="5" customWidth="1"/>
+    <col min="2" max="2" width="12.625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="14.125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="45.625" style="2" customWidth="1"/>
+    <col min="5" max="5" width="8.875" style="2"/>
     <col min="6" max="6" width="29.5" style="3" customWidth="1"/>
-    <col min="7" max="7" width="49.33203125" style="3" customWidth="1"/>
+    <col min="7" max="7" width="49.375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -1635,1408 +1643,1409 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="B2" s="4">
         <v>2026</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="F2" s="4"/>
       <c r="G2" s="25"/>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="B3" s="4">
         <v>2026</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="F3" s="4"/>
       <c r="G3" s="25"/>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B4" s="4">
         <v>2026</v>
       </c>
       <c r="C4" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>164</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>170</v>
-      </c>
       <c r="E4" s="4" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="F4" s="4"/>
       <c r="G4" s="25"/>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
-        <v>268</v>
+        <v>262</v>
       </c>
       <c r="B5" s="4">
         <v>2026</v>
       </c>
       <c r="C5" s="25" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D5" s="25" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="E5" s="25" t="s">
-        <v>270</v>
+        <v>264</v>
       </c>
       <c r="F5" s="4"/>
       <c r="G5" s="25"/>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B6" s="4">
         <v>2025</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="G6" s="23" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B7" s="4">
         <v>2024</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="E7" s="4"/>
       <c r="F7" s="4" t="s">
-        <v>177</v>
+        <v>171</v>
       </c>
       <c r="G7" s="23" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B8" s="4">
         <v>2023</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>178</v>
+        <v>172</v>
       </c>
       <c r="E8" s="4"/>
       <c r="F8" s="4" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="G8" s="23" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B9" s="4">
         <v>2023</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>179</v>
+        <v>173</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="25"/>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="B10" s="4">
         <v>2023</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="25"/>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="B11" s="5">
         <v>2023</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B12" s="4">
         <v>2022</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
       <c r="G12" s="25" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B13" s="4">
         <v>2022</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
       <c r="E13" s="4"/>
       <c r="F13" s="4"/>
       <c r="G13" s="25"/>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B14" s="4">
         <v>2022</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
       <c r="E14" s="4"/>
       <c r="F14" s="4"/>
       <c r="G14" s="25"/>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
       <c r="B15" s="4">
         <v>2022</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="E15" s="4"/>
       <c r="F15" s="4" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="G15" s="25" t="s">
-        <v>256</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B16" s="4">
         <v>2022</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="E16" s="4"/>
       <c r="F16" s="4" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
       <c r="B17" s="4">
         <v>2022</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="E17" s="4"/>
       <c r="F17" s="4"/>
       <c r="G17" s="25"/>
     </row>
-    <row r="18" spans="1:7">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18" s="25" t="s">
-        <v>262</v>
+        <v>256</v>
       </c>
       <c r="B18" s="4">
         <v>2021</v>
       </c>
       <c r="C18" s="25" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D18" s="25" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="E18" s="25" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="F18" s="25" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19" s="25" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="B19" s="4">
         <v>2021</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4"/>
       <c r="G19" s="23" t="s">
-        <v>251</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B20" s="18" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="G20" s="24" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="B21" s="18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G21" s="24" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="B22" s="18">
+        <v>2020</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="G22" s="24"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="B24" s="18" t="s">
         <v>48</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="C24" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G25" s="24" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="B26" s="20" t="s">
+        <v>230</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="G26" s="24" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="B27" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B28" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D28" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F20" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="G20" s="24" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
-      <c r="A21" s="8" t="s">
+    </row>
+    <row r="29" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+      <c r="A29" s="10" t="s">
+        <v>212</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="F29" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="10" t="s">
+        <v>213</v>
+      </c>
+      <c r="B30" s="20" t="s">
+        <v>52</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="B32" s="20">
+        <v>2010</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="9" t="s">
+        <v>188</v>
+      </c>
+      <c r="B33" s="20" t="s">
+        <v>54</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="G33" s="24" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="9" t="s">
+        <v>206</v>
+      </c>
+      <c r="B34" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="F34" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="9" t="s">
+        <v>216</v>
+      </c>
+      <c r="B35" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F35" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="B36" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="B38" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B39" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F39" s="3" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="B40" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A41" s="9" t="s">
         <v>208</v>
       </c>
-      <c r="B21" s="18" t="s">
-        <v>49</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="G21" s="24" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
-      <c r="A22" s="8" t="s">
+      <c r="B41" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="F41" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B42" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="B43" s="21" t="s">
+        <v>64</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="12" t="s">
         <v>209</v>
       </c>
-      <c r="B22" s="18" t="s">
-        <v>50</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D22" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
-      <c r="A23" s="8" t="s">
+      <c r="B44" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" ht="17.25" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="A45" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B45" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="13" t="s">
         <v>210</v>
-      </c>
-      <c r="B23" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>114</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
-      <c r="A24" s="9" t="s">
-        <v>211</v>
-      </c>
-      <c r="B24" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="C24" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D24" s="2" t="s">
-        <v>115</v>
-      </c>
-      <c r="G24" s="24" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
-      <c r="A25" s="9" t="s">
-        <v>234</v>
-      </c>
-      <c r="B25" s="20" t="s">
-        <v>236</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>193</v>
-      </c>
-      <c r="G25" s="24" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
-      <c r="A26" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="B26" s="20" t="s">
-        <v>237</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>167</v>
-      </c>
-      <c r="D26" s="2" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
-      <c r="A27" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="B27" s="20" t="s">
-        <v>53</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D27" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" ht="30">
-      <c r="A28" s="10" t="s">
-        <v>218</v>
-      </c>
-      <c r="B28" s="20" t="s">
-        <v>54</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D28" s="2" t="s">
-        <v>118</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>155</v>
-      </c>
-      <c r="G28" s="3" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
-      <c r="A29" s="10" t="s">
-        <v>219</v>
-      </c>
-      <c r="B29" s="20" t="s">
-        <v>55</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D29" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
-      <c r="A30" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="B30" s="20" t="s">
-        <v>56</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
-      <c r="A31" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="B31" s="20">
-        <v>2010</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
-      <c r="A32" s="9" t="s">
-        <v>194</v>
-      </c>
-      <c r="B32" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D32" s="2" t="s">
-        <v>121</v>
-      </c>
-      <c r="G32" s="24" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
-      <c r="A33" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="B33" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>122</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G33" s="3" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
-      <c r="A34" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="B34" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="C34" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="F34" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="G34" s="3" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
-      <c r="A35" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="B35" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
-      <c r="A36" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B36" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="F36" s="3" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
-      <c r="A37" s="9" t="s">
-        <v>195</v>
-      </c>
-      <c r="B37" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
-      <c r="A38" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="B38" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F38" s="3" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
-      <c r="A39" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="B39" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
-      <c r="A40" s="9" t="s">
-        <v>214</v>
-      </c>
-      <c r="B40" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="F40" s="3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7" ht="16" thickBot="1">
-      <c r="A41" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="B41" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7" ht="17" thickTop="1" thickBot="1">
-      <c r="A42" s="12" t="s">
-        <v>12</v>
-      </c>
-      <c r="B42" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7" ht="17" thickTop="1" thickBot="1">
-      <c r="A43" s="12" t="s">
-        <v>215</v>
-      </c>
-      <c r="B43" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="G43" s="3" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" ht="17" thickTop="1" thickBot="1">
-      <c r="A44" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B44" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D44" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" ht="16" thickTop="1">
-      <c r="A45" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B45" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D45" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7">
-      <c r="A46" s="13" t="s">
-        <v>216</v>
       </c>
       <c r="B46" s="22">
         <v>201012.08</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D46" s="2" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B47" s="22" t="s">
+        <v>67</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G47" s="24" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="B47" s="22" t="s">
+      <c r="B48" s="22" t="s">
+        <v>68</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" s="14" t="s">
+        <v>16</v>
+      </c>
+      <c r="B49" s="22" t="s">
+        <v>69</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B50" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B51" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="C47" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D47" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="G47" s="24" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7">
-      <c r="A48" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="B48" s="22" t="s">
+      <c r="C51" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A52" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="B52" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="C48" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7">
-      <c r="A49" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B49" s="22" t="s">
+      <c r="C52" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" s="14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B53" s="22" t="s">
         <v>73</v>
       </c>
-      <c r="C49" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F49" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="50" spans="1:7">
-      <c r="A50" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B50" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="C50" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D50" s="2" t="s">
-        <v>132</v>
-      </c>
-      <c r="G50" s="3" t="s">
-        <v>248</v>
-      </c>
-    </row>
-    <row r="51" spans="1:7">
-      <c r="A51" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B51" s="22" t="s">
-        <v>75</v>
-      </c>
-      <c r="C51" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D51" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="52" spans="1:7">
-      <c r="A52" s="14" t="s">
-        <v>217</v>
-      </c>
-      <c r="B52" s="22" t="s">
-        <v>76</v>
-      </c>
-      <c r="C52" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D52" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="53" spans="1:7">
-      <c r="A53" s="14" t="s">
+      <c r="C53" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" ht="27" x14ac:dyDescent="0.3">
+      <c r="A54" s="14" t="s">
         <v>20</v>
-      </c>
-      <c r="B53" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="C53" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="54" spans="1:7" ht="30">
-      <c r="A54" s="14" t="s">
-        <v>21</v>
       </c>
       <c r="B54" s="22">
         <v>2008</v>
       </c>
       <c r="C54" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="B55" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F55" s="3" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="B56" s="22" t="s">
+        <v>265</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="B57" s="22" t="s">
+        <v>75</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D57" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D54" s="6" t="s">
+      <c r="G57" s="24" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" s="14" t="s">
+        <v>218</v>
+      </c>
+      <c r="B58" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" s="14" t="s">
+        <v>24</v>
+      </c>
+      <c r="B59" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F59" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A60" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B60" s="22">
+        <v>1996</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="B61" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" s="14" t="s">
+        <v>219</v>
+      </c>
+      <c r="B62" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" s="14" t="s">
+        <v>27</v>
+      </c>
+      <c r="B63" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F63" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="B64" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A65" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="B65" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F65" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="G65" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="B66" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="F66" s="3" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A67" s="14" t="s">
+        <v>30</v>
+      </c>
+      <c r="B67" s="22" t="s">
+        <v>84</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="B68" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="C68" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D68" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F54" s="3" t="s">
-        <v>257</v>
-      </c>
-    </row>
-    <row r="55" spans="1:7">
-      <c r="A55" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="B55" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="C55" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D55" s="2" t="s">
+    </row>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A69" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="B69" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="C69" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D69" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="F69" s="3" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="B70" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="C70" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D70" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="F55" s="3" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="56" spans="1:7">
-      <c r="A56" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="B56" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="C56" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D56" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="57" spans="1:7">
-      <c r="A57" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B57" s="22" t="s">
-        <v>80</v>
-      </c>
-      <c r="C57" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D57" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="G57" s="24" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="58" spans="1:7">
-      <c r="A58" s="14" t="s">
-        <v>224</v>
-      </c>
-      <c r="B58" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="C58" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="59" spans="1:7">
-      <c r="A59" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="B59" s="22" t="s">
-        <v>82</v>
-      </c>
-      <c r="C59" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D59" s="2" t="s">
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="B71" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="C71" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D71" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" ht="40.5" x14ac:dyDescent="0.3">
+      <c r="A72" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="B72" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="C72" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D72" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="F59" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="60" spans="1:7">
-      <c r="A60" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="B60" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="C60" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D60" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="61" spans="1:7">
-      <c r="A61" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B61" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="C61" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D61" s="2" t="s">
+    </row>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A73" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="B73" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="C73" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D73" s="2" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="62" spans="1:7">
-      <c r="A62" s="14" t="s">
-        <v>225</v>
-      </c>
-      <c r="B62" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="C62" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D62" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="63" spans="1:7">
-      <c r="A63" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="B63" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="C63" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="F63" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="64" spans="1:7">
-      <c r="A64" s="14" t="s">
-        <v>226</v>
-      </c>
-      <c r="B64" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="C64" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D64" s="2" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="65" spans="1:7">
-      <c r="A65" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B65" s="22" t="s">
-        <v>88</v>
-      </c>
-      <c r="C65" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D65" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="F65" s="3" t="s">
-        <v>230</v>
-      </c>
-      <c r="G65" s="3" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="66" spans="1:7">
-      <c r="A66" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="B66" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="C66" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>140</v>
-      </c>
-      <c r="F66" s="3" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="67" spans="1:7">
-      <c r="A67" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B67" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="C67" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D67" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="68" spans="1:7">
-      <c r="A68" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="B68" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="C68" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D68" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7">
-      <c r="A69" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="B69" s="22" t="s">
-        <v>92</v>
-      </c>
-      <c r="C69" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D69" s="2" t="s">
-        <v>129</v>
-      </c>
-      <c r="F69" s="3" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7">
-      <c r="A70" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="B70" s="22" t="s">
-        <v>93</v>
-      </c>
-      <c r="C70" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D70" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7">
-      <c r="A71" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="B71" s="22" t="s">
-        <v>94</v>
-      </c>
-      <c r="C71" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D71" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" ht="45">
-      <c r="A72" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="B72" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="C72" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D72" s="6" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7">
-      <c r="A73" s="15" t="s">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A74" s="16" t="s">
         <v>37</v>
-      </c>
-      <c r="B73" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D73" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7">
-      <c r="A74" s="16" t="s">
-        <v>38</v>
       </c>
       <c r="B74" s="22">
         <v>200310</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D74" s="2" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B75" s="22">
         <v>200311</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D75" s="6" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="76" spans="1:7">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B76" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="C76" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="F76" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B76" s="22" t="s">
+      <c r="B77" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="C77" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D77" s="6" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A78" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B78" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="C78" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D78" s="2" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="B79" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="C79" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D79" s="6" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="80" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A80" s="16" t="s">
+        <v>272</v>
+      </c>
+      <c r="B80" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="C80" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="D80" s="2" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B81" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="C81" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D81" s="6" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" s="16" t="s">
+        <v>268</v>
+      </c>
+      <c r="B82" s="22" t="s">
         <v>97</v>
       </c>
-      <c r="C76" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="D76" s="2" t="s">
-        <v>147</v>
-      </c>
-      <c r="F76" s="3" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="77" spans="1:7">
-      <c r="A77" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="B77" s="22" t="s">
+      <c r="C82" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="B83" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="C77" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D77" s="6" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="78" spans="1:7">
-      <c r="A78" s="16" t="s">
-        <v>107</v>
-      </c>
-      <c r="B78" s="22" t="s">
-        <v>99</v>
-      </c>
-      <c r="C78" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D78" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="79" spans="1:7">
-      <c r="A79" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="B79" s="22" t="s">
+      <c r="C83" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C79" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D79" s="6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="80" spans="1:7">
-      <c r="A80" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="B80" s="22" t="s">
-        <v>101</v>
-      </c>
-      <c r="C80" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="D80" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4">
-      <c r="A81" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="B81" s="22" t="s">
-        <v>102</v>
-      </c>
-      <c r="C81" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="D81" s="6" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4">
-      <c r="A82" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="B82" s="22" t="s">
-        <v>103</v>
-      </c>
-      <c r="C82" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D82" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4">
-      <c r="A83" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="B83" s="22" t="s">
-        <v>104</v>
-      </c>
-      <c r="C83" s="2" t="s">
-        <v>106</v>
-      </c>
       <c r="D83" s="6" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="17" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B84" s="21">
         <v>1996</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D84" s="6" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" ht="16" thickBot="1">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="17" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B85" s="21">
         <v>1996</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>175</v>
+        <v>169</v>
       </c>
       <c r="D85" s="6" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" ht="16" thickTop="1">
-      <c r="A86" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B86" s="21">
-        <v>1996</v>
+        <v>222</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A86" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="B86" s="22">
+        <v>1994</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>109</v>
+        <v>146</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4">
-      <c r="A87" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="B87" s="22">
-        <v>1994</v>
+        <v>147</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A87" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="B87" s="5">
+        <v>1995</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>152</v>
+        <v>184</v>
       </c>
       <c r="D87" s="2" t="s">
-        <v>153</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="G8" r:id="rId1" xr:uid="{EE7197D7-D691-E942-A734-EF468BD5BEC1}"/>
-    <hyperlink ref="G25" r:id="rId2" xr:uid="{913ECA8B-EAA8-5043-A4E7-4DAA8CCBE80B}"/>
+    <hyperlink ref="G26" r:id="rId2" xr:uid="{913ECA8B-EAA8-5043-A4E7-4DAA8CCBE80B}"/>
     <hyperlink ref="G57" r:id="rId3" xr:uid="{17AFEC1C-5E7A-6D42-BBF1-3EED48E7F950}"/>
-    <hyperlink ref="G24" r:id="rId4" xr:uid="{9692D92D-6D8E-F04F-A1A7-FED686B2B67F}"/>
+    <hyperlink ref="G25" r:id="rId4" xr:uid="{9692D92D-6D8E-F04F-A1A7-FED686B2B67F}"/>
     <hyperlink ref="G21" r:id="rId5" xr:uid="{7566423B-7ABB-C245-95BF-210A8C3D0F5F}"/>
     <hyperlink ref="G47" r:id="rId6" xr:uid="{CDAA89B4-C6EA-A142-9137-71CDCACD6A61}"/>
-    <hyperlink ref="G32" r:id="rId7" xr:uid="{ACC8F633-2D7C-7349-98A3-F522A6F9C03E}"/>
+    <hyperlink ref="G33" r:id="rId7" xr:uid="{ACC8F633-2D7C-7349-98A3-F522A6F9C03E}"/>
     <hyperlink ref="G16" r:id="rId8" xr:uid="{A658E596-88B1-E443-8DA8-ACE3D30929A5}"/>
     <hyperlink ref="G19" r:id="rId9" xr:uid="{C5474A65-32DB-8345-8D9F-0EBA5F582518}"/>
     <hyperlink ref="G6" r:id="rId10" xr:uid="{27800473-DF59-D24F-AD62-DB892F72A562}"/>

</xml_diff>